<commit_message>
chore(checkpoint): UI 系统 P1 收口 + 工具链/文档同步
UI 系统 P1-5/P1-6（P1 收口）：
- 新增 ui.contract / ui.contract-diff / ui.widget-manifest / ui.page-manifest 四个 Hub/CLI 动作；
  UiContractBatch 批量生成（表只读一次、按 prefab 去重、常驻壳 UIMain 跳过并告警、多行取首行）
- 起页 UiPageScaffold.Create 成功后自动对账页面清单（失败只记日志）
- 试点页 Page_Login：Txt_Title/Txt_GuestLogin/Txt_Settings 改 LTextKeyRef，Lua 删除三处静态写
- 生成物基线入库：11 份页面契约 + 控件清单 + 页面清单（contractPresent 转真）

同批包含：工具链 Hub 合并（新建页/UI 制作）与清单索引同步、现行 UI 系统文档体系与旧体系归档、
以及工作区内其他在途线（TPS/表现/DevHUD 等）改动，一并作为检查点入库。

验证：L1 1819 · Doc 0 violation · L2 meta 14216 · wf verify 20/20（UI 新夹具 8/8，先红 5/5）
</commit_message>
<xml_diff>
--- a/Luban/Data/#contententry.xlsx
+++ b/Luban/Data/#contententry.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,21 +479,6 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>内容处理器Lua路径(Content.处理器名)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>demo_entry</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Content.DemoEntry</t>
         </is>
       </c>
     </row>

</xml_diff>